<commit_message>
Release v1.1.10: multi-MQTT publish, scan/publish interval split, and history/Android fixes.
Separate MQTT publish cadence from PLC scan, support multiple broker targets with simultaneous send, and patch config/lines with MQTT目标 sheets.
</commit_message>
<xml_diff>
--- a/config/lines/C型火焰复合机.xlsx
+++ b/config/lines/C型火焰复合机.xlsx
@@ -11,6 +11,7 @@
     <x:sheet name="字段映射" sheetId="3" r:id="rId4"/>
     <x:sheet name="点表" sheetId="4" r:id="rId5"/>
     <x:sheet name="显示分组说明" sheetId="5" r:id="rId6"/>
+    <x:sheet name="MQTT目标" sheetId="6" r:id="rId9"/>
   </x:sheets>
   <x:definedNames/>
   <x:calcPr calcId="125725"/>
@@ -335,42 +336,81 @@
     <x:t>车速</x:t>
   </x:si>
   <x:si>
+    <x:t>hmwrzl</x:t>
+  </x:si>
+  <x:si>
     <x:t>海绵喂入张力</x:t>
   </x:si>
   <x:si>
+    <x:t>sjj</x:t>
+  </x:si>
+  <x:si>
     <x:t>上夹距</x:t>
   </x:si>
   <x:si>
+    <x:t>xjj</x:t>
+  </x:si>
+  <x:si>
     <x:t>下夹距</x:t>
   </x:si>
   <x:si>
+    <x:t>shkjjl</x:t>
+  </x:si>
+  <x:si>
     <x:t>上火口距离</x:t>
   </x:si>
   <x:si>
+    <x:t>xhkjjl</x:t>
+  </x:si>
+  <x:si>
     <x:t>下火口距离</x:t>
   </x:si>
   <x:si>
+    <x:t>smqll</x:t>
+  </x:si>
+  <x:si>
     <x:t>上煤气流量</x:t>
   </x:si>
   <x:si>
+    <x:t>xmqll</x:t>
+  </x:si>
+  <x:si>
     <x:t>下煤气流量</x:t>
   </x:si>
   <x:si>
+    <x:t>cpwrsd</x:t>
+  </x:si>
+  <x:si>
     <x:t>成品喂入速度</x:t>
   </x:si>
   <x:si>
+    <x:t>sjqysd</x:t>
+  </x:si>
+  <x:si>
     <x:t>收卷牵引速度</x:t>
   </x:si>
   <x:si>
+    <x:t>sjxs</x:t>
+  </x:si>
+  <x:si>
     <x:t>收卷系数</x:t>
   </x:si>
   <x:si>
+    <x:t>qdjj</x:t>
+  </x:si>
+  <x:si>
     <x:t>切刀间距</x:t>
   </x:si>
   <x:si>
+    <x:t>mf</x:t>
+  </x:si>
+  <x:si>
     <x:t>门幅</x:t>
   </x:si>
   <x:si>
+    <x:t>hd</x:t>
+  </x:si>
+  <x:si>
     <x:t>厚度</x:t>
   </x:si>
   <x:si>
@@ -530,43 +570,37 @@
     <x:t>在「点表」工作表的「显示分组」列填写上表分组名称；留空则程序按数据类型自动推断。</x:t>
   </x:si>
   <x:si>
-    <x:t>hmwrzl</x:t>
-  </x:si>
-  <x:si>
-    <x:t>sjj</x:t>
-  </x:si>
-  <x:si>
-    <x:t>xjj</x:t>
-  </x:si>
-  <x:si>
-    <x:t>shkjjl</x:t>
-  </x:si>
-  <x:si>
-    <x:t>xhkjjl</x:t>
-  </x:si>
-  <x:si>
-    <x:t>smqll</x:t>
-  </x:si>
-  <x:si>
-    <x:t>xmqll</x:t>
-  </x:si>
-  <x:si>
-    <x:t>cpwrsd</x:t>
-  </x:si>
-  <x:si>
-    <x:t>sjqysd</x:t>
-  </x:si>
-  <x:si>
-    <x:t>sjxs</x:t>
-  </x:si>
-  <x:si>
-    <x:t>qdjj</x:t>
-  </x:si>
-  <x:si>
-    <x:t>mf</x:t>
-  </x:si>
-  <x:si>
-    <x:t>hd</x:t>
+    <x:t>Broker</x:t>
+  </x:si>
+  <x:si>
+    <x:t>端口</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ClientId</x:t>
+  </x:si>
+  <x:si>
+    <x:t>用户名</x:t>
+  </x:si>
+  <x:si>
+    <x:t>密码</x:t>
+  </x:si>
+  <x:si>
+    <x:t>TLS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>QoS</x:t>
+  </x:si>
+  <x:si>
+    <x:t>主题</x:t>
+  </x:si>
+  <x:si>
+    <x:t>ID</x:t>
+  </x:si>
+  <x:si>
+    <x:t>默认</x:t>
+  </x:si>
+  <x:si>
+    <x:t>4cc2730287d24d0eb035d4e6da9f6a45</x:t>
   </x:si>
 </x:sst>
 </file>
@@ -1427,106 +1461,106 @@
     </x:row>
     <x:row r="4" spans="1:2">
       <x:c r="A4" s="0" t="s">
-        <x:v>170</x:v>
+        <x:v>105</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>106</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:2">
       <x:c r="A5" s="0" t="s">
-        <x:v>171</x:v>
+        <x:v>107</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>108</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:2">
       <x:c r="A6" s="0" t="s">
-        <x:v>172</x:v>
+        <x:v>109</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>110</x:v>
       </x:c>
     </x:row>
     <x:row r="7" spans="1:2">
       <x:c r="A7" s="0" t="s">
-        <x:v>173</x:v>
+        <x:v>111</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>108</x:v>
+        <x:v>112</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:2">
       <x:c r="A8" s="0" t="s">
-        <x:v>174</x:v>
+        <x:v>113</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>109</x:v>
+        <x:v>114</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:2">
       <x:c r="A9" s="0" t="s">
-        <x:v>175</x:v>
+        <x:v>115</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>116</x:v>
       </x:c>
     </x:row>
     <x:row r="10" spans="1:2">
       <x:c r="A10" s="0" t="s">
-        <x:v>176</x:v>
+        <x:v>117</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>118</x:v>
       </x:c>
     </x:row>
     <x:row r="11" spans="1:2">
       <x:c r="A11" s="0" t="s">
-        <x:v>177</x:v>
+        <x:v>119</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
-        <x:v>112</x:v>
+        <x:v>120</x:v>
       </x:c>
     </x:row>
     <x:row r="12" spans="1:2">
       <x:c r="A12" s="0" t="s">
-        <x:v>178</x:v>
+        <x:v>121</x:v>
       </x:c>
       <x:c r="B12" s="0" t="s">
-        <x:v>113</x:v>
+        <x:v>122</x:v>
       </x:c>
     </x:row>
     <x:row r="13" spans="1:2">
       <x:c r="A13" s="0" t="s">
-        <x:v>179</x:v>
+        <x:v>123</x:v>
       </x:c>
       <x:c r="B13" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>124</x:v>
       </x:c>
     </x:row>
     <x:row r="14" spans="1:2">
       <x:c r="A14" s="0" t="s">
-        <x:v>180</x:v>
+        <x:v>125</x:v>
       </x:c>
       <x:c r="B14" s="0" t="s">
-        <x:v>115</x:v>
+        <x:v>126</x:v>
       </x:c>
     </x:row>
     <x:row r="15" spans="1:2">
       <x:c r="A15" s="0" t="s">
-        <x:v>181</x:v>
+        <x:v>127</x:v>
       </x:c>
       <x:c r="B15" s="0" t="s">
-        <x:v>116</x:v>
+        <x:v>128</x:v>
       </x:c>
     </x:row>
     <x:row r="16" spans="1:2">
       <x:c r="A16" s="0" t="s">
-        <x:v>182</x:v>
+        <x:v>129</x:v>
       </x:c>
       <x:c r="B16" s="0" t="s">
-        <x:v>117</x:v>
+        <x:v>130</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -1560,43 +1594,43 @@
   <x:sheetData>
     <x:row r="1" spans="1:13" s="1" customFormat="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>118</x:v>
+        <x:v>131</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
-        <x:v>119</x:v>
+        <x:v>132</x:v>
       </x:c>
       <x:c r="C1" s="1" t="s">
-        <x:v>120</x:v>
+        <x:v>133</x:v>
       </x:c>
       <x:c r="D1" s="1" t="s">
-        <x:v>121</x:v>
+        <x:v>134</x:v>
       </x:c>
       <x:c r="E1" s="1" t="s">
-        <x:v>122</x:v>
+        <x:v>135</x:v>
       </x:c>
       <x:c r="F1" s="1" t="s">
-        <x:v>123</x:v>
+        <x:v>136</x:v>
       </x:c>
       <x:c r="G1" s="1" t="s">
-        <x:v>124</x:v>
+        <x:v>137</x:v>
       </x:c>
       <x:c r="H1" s="1" t="s">
-        <x:v>125</x:v>
+        <x:v>138</x:v>
       </x:c>
       <x:c r="I1" s="1" t="s">
         <x:v>35</x:v>
       </x:c>
       <x:c r="J1" s="1" t="s">
-        <x:v>126</x:v>
+        <x:v>139</x:v>
       </x:c>
       <x:c r="K1" s="1" t="s">
-        <x:v>127</x:v>
+        <x:v>140</x:v>
       </x:c>
       <x:c r="L1" s="1" t="s">
-        <x:v>128</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="M1" s="1" t="s">
-        <x:v>129</x:v>
+        <x:v>142</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:13">
@@ -1604,19 +1638,19 @@
         <x:v>102</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>130</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>131</x:v>
+        <x:v>144</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>132</x:v>
+        <x:v>145</x:v>
       </x:c>
       <x:c r="E2" s="0" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="F2" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="G2" s="0" t="s">
         <x:v>38</x:v>
@@ -1634,7 +1668,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L2" s="0" t="s">
-        <x:v>134</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="M2" s="0" t="s">
         <x:v>56</x:v>
@@ -1645,19 +1679,19 @@
         <x:v>104</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>130</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>135</x:v>
+        <x:v>148</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E3" s="0" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="F3" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="G3" s="0" t="s">
         <x:v>38</x:v>
@@ -1675,7 +1709,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L3" s="0" t="s">
-        <x:v>137</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="M3" s="0" t="s">
         <x:v>56</x:v>
@@ -1683,22 +1717,22 @@
     </x:row>
     <x:row r="4" spans="1:13">
       <x:c r="A4" s="0" t="s">
-        <x:v>105</x:v>
+        <x:v>106</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>130</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>138</x:v>
+        <x:v>151</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E4" s="0" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="F4" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="G4" s="0" t="s">
         <x:v>38</x:v>
@@ -1716,7 +1750,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L4" s="0" t="s">
-        <x:v>137</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="M4" s="0" t="s">
         <x:v>56</x:v>
@@ -1724,22 +1758,22 @@
     </x:row>
     <x:row r="5" spans="1:13">
       <x:c r="A5" s="0" t="s">
-        <x:v>106</x:v>
+        <x:v>108</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>130</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>139</x:v>
+        <x:v>152</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E5" s="0" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="F5" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="G5" s="0" t="s">
         <x:v>38</x:v>
@@ -1757,7 +1791,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L5" s="0" t="s">
-        <x:v>137</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="M5" s="0" t="s">
         <x:v>56</x:v>
@@ -1765,22 +1799,22 @@
     </x:row>
     <x:row r="6" spans="1:13">
       <x:c r="A6" s="0" t="s">
-        <x:v>107</x:v>
+        <x:v>110</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>130</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>140</x:v>
+        <x:v>153</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E6" s="0" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="F6" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="G6" s="0" t="s">
         <x:v>38</x:v>
@@ -1798,7 +1832,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L6" s="0" t="s">
-        <x:v>137</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="M6" s="0" t="s">
         <x:v>56</x:v>
@@ -1806,22 +1840,22 @@
     </x:row>
     <x:row r="7" spans="1:13">
       <x:c r="A7" s="0" t="s">
-        <x:v>108</x:v>
+        <x:v>112</x:v>
       </x:c>
       <x:c r="B7" s="0" t="s">
-        <x:v>130</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="C7" s="0" t="s">
-        <x:v>141</x:v>
+        <x:v>154</x:v>
       </x:c>
       <x:c r="D7" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E7" s="0" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="F7" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="G7" s="0" t="s">
         <x:v>38</x:v>
@@ -1839,7 +1873,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L7" s="0" t="s">
-        <x:v>137</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="M7" s="0" t="s">
         <x:v>56</x:v>
@@ -1847,22 +1881,22 @@
     </x:row>
     <x:row r="8" spans="1:13">
       <x:c r="A8" s="0" t="s">
-        <x:v>109</x:v>
+        <x:v>114</x:v>
       </x:c>
       <x:c r="B8" s="0" t="s">
-        <x:v>130</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="C8" s="0" t="s">
-        <x:v>142</x:v>
+        <x:v>155</x:v>
       </x:c>
       <x:c r="D8" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E8" s="0" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="F8" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="G8" s="0" t="s">
         <x:v>38</x:v>
@@ -1880,7 +1914,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L8" s="0" t="s">
-        <x:v>137</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="M8" s="0" t="s">
         <x:v>56</x:v>
@@ -1888,22 +1922,22 @@
     </x:row>
     <x:row r="9" spans="1:13">
       <x:c r="A9" s="0" t="s">
-        <x:v>110</x:v>
+        <x:v>116</x:v>
       </x:c>
       <x:c r="B9" s="0" t="s">
-        <x:v>130</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="C9" s="0" t="s">
-        <x:v>143</x:v>
+        <x:v>156</x:v>
       </x:c>
       <x:c r="D9" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E9" s="0" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="F9" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="G9" s="0" t="s">
         <x:v>38</x:v>
@@ -1921,7 +1955,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L9" s="0" t="s">
-        <x:v>137</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="M9" s="0" t="s">
         <x:v>56</x:v>
@@ -1929,22 +1963,22 @@
     </x:row>
     <x:row r="10" spans="1:13">
       <x:c r="A10" s="0" t="s">
-        <x:v>111</x:v>
+        <x:v>118</x:v>
       </x:c>
       <x:c r="B10" s="0" t="s">
-        <x:v>130</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="C10" s="0" t="s">
-        <x:v>144</x:v>
+        <x:v>157</x:v>
       </x:c>
       <x:c r="D10" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E10" s="0" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="F10" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="G10" s="0" t="s">
         <x:v>38</x:v>
@@ -1962,7 +1996,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L10" s="0" t="s">
-        <x:v>137</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="M10" s="0" t="s">
         <x:v>56</x:v>
@@ -1970,22 +2004,22 @@
     </x:row>
     <x:row r="11" spans="1:13">
       <x:c r="A11" s="0" t="s">
-        <x:v>112</x:v>
+        <x:v>120</x:v>
       </x:c>
       <x:c r="B11" s="0" t="s">
-        <x:v>130</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="C11" s="0" t="s">
-        <x:v>145</x:v>
+        <x:v>158</x:v>
       </x:c>
       <x:c r="D11" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E11" s="0" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="F11" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="G11" s="0" t="s">
         <x:v>38</x:v>
@@ -2003,7 +2037,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L11" s="0" t="s">
-        <x:v>137</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="M11" s="0" t="s">
         <x:v>56</x:v>
@@ -2011,22 +2045,22 @@
     </x:row>
     <x:row r="12" spans="1:13">
       <x:c r="A12" s="0" t="s">
-        <x:v>113</x:v>
+        <x:v>122</x:v>
       </x:c>
       <x:c r="B12" s="0" t="s">
-        <x:v>130</x:v>
+        <x:v>143</x:v>
       </x:c>
       <x:c r="C12" s="0" t="s">
+        <x:v>159</x:v>
+      </x:c>
+      <x:c r="D12" s="0" t="s">
+        <x:v>149</x:v>
+      </x:c>
+      <x:c r="E12" s="0" t="s">
+        <x:v>84</x:v>
+      </x:c>
+      <x:c r="F12" s="0" t="s">
         <x:v>146</x:v>
-      </x:c>
-      <x:c r="D12" s="0" t="s">
-        <x:v>136</x:v>
-      </x:c>
-      <x:c r="E12" s="0" t="s">
-        <x:v>84</x:v>
-      </x:c>
-      <x:c r="F12" s="0" t="s">
-        <x:v>133</x:v>
       </x:c>
       <x:c r="G12" s="0" t="s">
         <x:v>38</x:v>
@@ -2044,7 +2078,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L12" s="0" t="s">
-        <x:v>137</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="M12" s="0" t="s">
         <x:v>56</x:v>
@@ -2052,22 +2086,22 @@
     </x:row>
     <x:row r="13" spans="1:13">
       <x:c r="A13" s="0" t="s">
-        <x:v>114</x:v>
+        <x:v>124</x:v>
       </x:c>
       <x:c r="B13" s="0" t="s">
-        <x:v>147</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="C13" s="0" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="D13" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E13" s="0" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="F13" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="G13" s="0" t="s">
         <x:v>38</x:v>
@@ -2085,7 +2119,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L13" s="0" t="s">
-        <x:v>148</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="M13" s="0" t="s">
         <x:v>56</x:v>
@@ -2093,22 +2127,22 @@
     </x:row>
     <x:row r="14" spans="1:13">
       <x:c r="A14" s="0" t="s">
-        <x:v>115</x:v>
+        <x:v>126</x:v>
       </x:c>
       <x:c r="B14" s="0" t="s">
-        <x:v>147</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="C14" s="0" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="D14" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E14" s="0" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="F14" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="G14" s="0" t="s">
         <x:v>38</x:v>
@@ -2126,7 +2160,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L14" s="0" t="s">
-        <x:v>148</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="M14" s="0" t="s">
         <x:v>56</x:v>
@@ -2134,22 +2168,22 @@
     </x:row>
     <x:row r="15" spans="1:13">
       <x:c r="A15" s="0" t="s">
-        <x:v>116</x:v>
+        <x:v>128</x:v>
       </x:c>
       <x:c r="B15" s="0" t="s">
-        <x:v>147</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="C15" s="0" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="D15" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E15" s="0" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="F15" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="G15" s="0" t="s">
         <x:v>38</x:v>
@@ -2167,7 +2201,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L15" s="0" t="s">
-        <x:v>148</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="M15" s="0" t="s">
         <x:v>56</x:v>
@@ -2175,22 +2209,22 @@
     </x:row>
     <x:row r="16" spans="1:13">
       <x:c r="A16" s="0" t="s">
-        <x:v>117</x:v>
+        <x:v>130</x:v>
       </x:c>
       <x:c r="B16" s="0" t="s">
-        <x:v>147</x:v>
+        <x:v>160</x:v>
       </x:c>
       <x:c r="C16" s="0" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="D16" s="0" t="s">
-        <x:v>136</x:v>
+        <x:v>149</x:v>
       </x:c>
       <x:c r="E16" s="0" t="s">
         <x:v>84</x:v>
       </x:c>
       <x:c r="F16" s="0" t="s">
-        <x:v>133</x:v>
+        <x:v>146</x:v>
       </x:c>
       <x:c r="G16" s="0" t="s">
         <x:v>38</x:v>
@@ -2208,7 +2242,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="L16" s="0" t="s">
-        <x:v>148</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="M16" s="0" t="s">
         <x:v>56</x:v>
@@ -2239,96 +2273,195 @@
   <x:sheetData>
     <x:row r="1" spans="1:4" s="1" customFormat="1">
       <x:c r="A1" s="1" t="s">
-        <x:v>128</x:v>
+        <x:v>141</x:v>
       </x:c>
       <x:c r="B1" s="1" t="s">
         <x:v>2</x:v>
       </x:c>
       <x:c r="C1" s="1" t="s">
-        <x:v>149</x:v>
+        <x:v>162</x:v>
       </x:c>
       <x:c r="D1" s="1" t="s">
-        <x:v>150</x:v>
+        <x:v>163</x:v>
       </x:c>
     </x:row>
     <x:row r="2" spans="1:4">
       <x:c r="A2" s="0" t="s">
-        <x:v>134</x:v>
+        <x:v>147</x:v>
       </x:c>
       <x:c r="B2" s="0" t="s">
-        <x:v>151</x:v>
+        <x:v>164</x:v>
       </x:c>
       <x:c r="C2" s="0" t="s">
-        <x:v>152</x:v>
+        <x:v>165</x:v>
       </x:c>
       <x:c r="D2" s="0" t="s">
-        <x:v>153</x:v>
+        <x:v>166</x:v>
       </x:c>
     </x:row>
     <x:row r="3" spans="1:4">
       <x:c r="A3" s="0" t="s">
-        <x:v>154</x:v>
+        <x:v>167</x:v>
       </x:c>
       <x:c r="B3" s="0" t="s">
-        <x:v>155</x:v>
+        <x:v>168</x:v>
       </x:c>
       <x:c r="C3" s="0" t="s">
-        <x:v>156</x:v>
+        <x:v>169</x:v>
       </x:c>
       <x:c r="D3" s="0" t="s">
-        <x:v>157</x:v>
+        <x:v>170</x:v>
       </x:c>
     </x:row>
     <x:row r="4" spans="1:4">
       <x:c r="A4" s="0" t="s">
-        <x:v>137</x:v>
+        <x:v>150</x:v>
       </x:c>
       <x:c r="B4" s="0" t="s">
-        <x:v>158</x:v>
+        <x:v>171</x:v>
       </x:c>
       <x:c r="C4" s="0" t="s">
-        <x:v>159</x:v>
+        <x:v>172</x:v>
       </x:c>
       <x:c r="D4" s="0" t="s">
-        <x:v>160</x:v>
+        <x:v>173</x:v>
       </x:c>
     </x:row>
     <x:row r="5" spans="1:4">
       <x:c r="A5" s="0" t="s">
-        <x:v>148</x:v>
+        <x:v>161</x:v>
       </x:c>
       <x:c r="B5" s="0" t="s">
-        <x:v>161</x:v>
+        <x:v>174</x:v>
       </x:c>
       <x:c r="C5" s="0" t="s">
-        <x:v>162</x:v>
+        <x:v>175</x:v>
       </x:c>
       <x:c r="D5" s="0" t="s">
-        <x:v>163</x:v>
+        <x:v>176</x:v>
       </x:c>
     </x:row>
     <x:row r="6" spans="1:4">
       <x:c r="A6" s="0" t="s">
-        <x:v>164</x:v>
+        <x:v>177</x:v>
       </x:c>
       <x:c r="B6" s="0" t="s">
-        <x:v>165</x:v>
+        <x:v>178</x:v>
       </x:c>
       <x:c r="C6" s="0" t="s">
-        <x:v>166</x:v>
+        <x:v>179</x:v>
       </x:c>
       <x:c r="D6" s="0" t="s">
-        <x:v>167</x:v>
+        <x:v>180</x:v>
       </x:c>
     </x:row>
     <x:row r="8" spans="1:4">
       <x:c r="A8" s="0" t="s">
-        <x:v>168</x:v>
+        <x:v>181</x:v>
       </x:c>
     </x:row>
     <x:row r="9" spans="1:4">
       <x:c r="A9" s="0" t="s">
-        <x:v>169</x:v>
+        <x:v>182</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:printOptions horizontalCentered="0" verticalCentered="0" headings="0" gridLines="0"/>
+  <x:pageMargins left="0.75" right="0.75" top="0.75" bottom="0.5" header="0.5" footer="0.75"/>
+  <x:pageSetup paperSize="1" scale="100" pageOrder="downThenOver" orientation="default" blackAndWhite="0" draft="0" cellComments="none" errors="displayed"/>
+  <x:headerFooter/>
+  <x:tableParts count="0"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x14ac">
+  <x:sheetPr>
+    <x:outlinePr summaryBelow="1" summaryRight="1"/>
+  </x:sheetPr>
+  <x:dimension ref="A1:K2"/>
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="2" width="2.996339" style="0" customWidth="1"/>
+    <x:col min="3" max="3" width="13.282054" style="0" customWidth="1"/>
+    <x:col min="4" max="4" width="4.996339" style="0" customWidth="1"/>
+    <x:col min="5" max="5" width="7.853482" style="0" customWidth="1"/>
+    <x:col min="6" max="6" width="6.424911" style="0" customWidth="1"/>
+    <x:col min="7" max="7" width="11.853482" style="0" customWidth="1"/>
+    <x:col min="8" max="8" width="3.853482" style="0" customWidth="1"/>
+    <x:col min="9" max="9" width="4.567768" style="0" customWidth="1"/>
+    <x:col min="10" max="10" width="32.567768" style="0" customWidth="1"/>
+    <x:col min="11" max="11" width="34.710625" style="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" spans="1:11" s="1" customFormat="1">
+      <x:c r="A1" s="1" t="s">
+        <x:v>131</x:v>
+      </x:c>
+      <x:c r="B1" s="1" t="s">
+        <x:v>137</x:v>
+      </x:c>
+      <x:c r="C1" s="1" t="s">
+        <x:v>183</x:v>
+      </x:c>
+      <x:c r="D1" s="1" t="s">
+        <x:v>184</x:v>
+      </x:c>
+      <x:c r="E1" s="1" t="s">
+        <x:v>185</x:v>
+      </x:c>
+      <x:c r="F1" s="1" t="s">
+        <x:v>186</x:v>
+      </x:c>
+      <x:c r="G1" s="1" t="s">
+        <x:v>187</x:v>
+      </x:c>
+      <x:c r="H1" s="1" t="s">
+        <x:v>188</x:v>
+      </x:c>
+      <x:c r="I1" s="1" t="s">
+        <x:v>189</x:v>
+      </x:c>
+      <x:c r="J1" s="1" t="s">
+        <x:v>190</x:v>
+      </x:c>
+      <x:c r="K1" s="1" t="s">
+        <x:v>191</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2" spans="1:11">
+      <x:c r="A2" s="0" t="s">
+        <x:v>192</x:v>
+      </x:c>
+      <x:c r="B2" s="0" t="s">
+        <x:v>38</x:v>
+      </x:c>
+      <x:c r="C2" s="0" t="s">
+        <x:v>41</x:v>
+      </x:c>
+      <x:c r="D2" s="0">
+        <x:v>1888</x:v>
+      </x:c>
+      <x:c r="E2" s="0" t="s">
+        <x:v>47</x:v>
+      </x:c>
+      <x:c r="F2" s="0" t="s">
+        <x:v>50</x:v>
+      </x:c>
+      <x:c r="G2" s="0" t="s">
+        <x:v>53</x:v>
+      </x:c>
+      <x:c r="H2" s="0" t="s">
+        <x:v>56</x:v>
+      </x:c>
+      <x:c r="I2" s="0">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="J2" s="0" t="s">
+        <x:v>61</x:v>
+      </x:c>
+      <x:c r="K2" s="0" t="s">
+        <x:v>193</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Release v1.1.10-r4: S7 test line, resilient PLC/config handling, and log export.
Add S7 test line Excel and catalog; improve S7 connect/read errors and per-tag reads. Load config without crashing UI/service; async line switch and log bundle export scripts.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/config/lines/C型火焰复合机.xlsx
+++ b/config/lines/C型火焰复合机.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="14400" windowHeight="11760"/>
+    <workbookView windowWidth="15120" windowHeight="11760"/>
   </bookViews>
   <sheets>
     <sheet name="配置" sheetId="1" r:id="rId1"/>
@@ -153,100 +153,100 @@
     <t>使用模拟数据</t>
   </si>
   <si>
+    <t>否</t>
+  </si>
+  <si>
+    <t>UseSimulator</t>
+  </si>
+  <si>
+    <t>MQTT_Broker</t>
+  </si>
+  <si>
+    <t>192.168.16.18</t>
+  </si>
+  <si>
+    <t>MqttHost</t>
+  </si>
+  <si>
+    <t>MQTT端口</t>
+  </si>
+  <si>
+    <t>1888</t>
+  </si>
+  <si>
+    <t>MqttPort</t>
+  </si>
+  <si>
+    <t>MQTT_ClientId</t>
+  </si>
+  <si>
+    <t>CYHYFJ</t>
+  </si>
+  <si>
+    <t>MqttClientId</t>
+  </si>
+  <si>
+    <t>MQTT_用户名</t>
+  </si>
+  <si>
+    <t>hg_iot</t>
+  </si>
+  <si>
+    <t>MqttUsername</t>
+  </si>
+  <si>
+    <t>MQTT_密码</t>
+  </si>
+  <si>
+    <t>Hg@Iot2026</t>
+  </si>
+  <si>
+    <t>MqttPassword</t>
+  </si>
+  <si>
+    <t>MQTT_TLS</t>
+  </si>
+  <si>
+    <t>MqttUseTls</t>
+  </si>
+  <si>
+    <t>MQTT_QoS</t>
+  </si>
+  <si>
+    <t>MqttQos</t>
+  </si>
+  <si>
+    <t>MQTT发布主题</t>
+  </si>
+  <si>
+    <t>/RRJFHJ/CYHYFJ/properties/report</t>
+  </si>
+  <si>
+    <t>MqttTopic</t>
+  </si>
+  <si>
+    <t>订阅主题</t>
+  </si>
+  <si>
+    <t>/RRJFHJ/XHRRJFHJ/properties/report;/RRJFHJ/HDRRJFHJ/properties/report</t>
+  </si>
+  <si>
+    <t>SubscribeTopics</t>
+  </si>
+  <si>
+    <t>运行模式</t>
+  </si>
+  <si>
+    <t>采集模式</t>
+  </si>
+  <si>
+    <t>OperationMode</t>
+  </si>
+  <si>
+    <t>开机自动启动</t>
+  </si>
+  <si>
     <t>是</t>
-  </si>
-  <si>
-    <t>UseSimulator</t>
-  </si>
-  <si>
-    <t>MQTT_Broker</t>
-  </si>
-  <si>
-    <t>192.168.16.18</t>
-  </si>
-  <si>
-    <t>MqttHost</t>
-  </si>
-  <si>
-    <t>MQTT端口</t>
-  </si>
-  <si>
-    <t>1888</t>
-  </si>
-  <si>
-    <t>MqttPort</t>
-  </si>
-  <si>
-    <t>MQTT_ClientId</t>
-  </si>
-  <si>
-    <t>CYHYFJ</t>
-  </si>
-  <si>
-    <t>MqttClientId</t>
-  </si>
-  <si>
-    <t>MQTT_用户名</t>
-  </si>
-  <si>
-    <t>hg_iot</t>
-  </si>
-  <si>
-    <t>MqttUsername</t>
-  </si>
-  <si>
-    <t>MQTT_密码</t>
-  </si>
-  <si>
-    <t>Hg@Iot2026</t>
-  </si>
-  <si>
-    <t>MqttPassword</t>
-  </si>
-  <si>
-    <t>MQTT_TLS</t>
-  </si>
-  <si>
-    <t>否</t>
-  </si>
-  <si>
-    <t>MqttUseTls</t>
-  </si>
-  <si>
-    <t>MQTT_QoS</t>
-  </si>
-  <si>
-    <t>MqttQos</t>
-  </si>
-  <si>
-    <t>MQTT发布主题</t>
-  </si>
-  <si>
-    <t>/RRJFHJ/CYHYFJ/properties/report</t>
-  </si>
-  <si>
-    <t>MqttTopic</t>
-  </si>
-  <si>
-    <t>订阅主题</t>
-  </si>
-  <si>
-    <t>/RRJFHJ/XHRRJFHJ/properties/report;/RRJFHJ/HDRRJFHJ/properties/report</t>
-  </si>
-  <si>
-    <t>SubscribeTopics</t>
-  </si>
-  <si>
-    <t>运行模式</t>
-  </si>
-  <si>
-    <t>采集模式</t>
-  </si>
-  <si>
-    <t>OperationMode</t>
-  </si>
-  <si>
-    <t>开机自动启动</t>
   </si>
   <si>
     <t>StartWithWindows</t>
@@ -628,7 +628,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="22">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -640,6 +640,12 @@
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="宋体"/>
       <charset val="134"/>
     </font>
     <font>
@@ -1097,154 +1103,155 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
-    <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1960,7 +1967,7 @@
       <c r="A14" t="s">
         <v>37</v>
       </c>
-      <c r="B14" t="s">
+      <c r="B14" s="2" t="s">
         <v>38</v>
       </c>
       <c r="C14" t="s">
@@ -2027,62 +2034,62 @@
         <v>55</v>
       </c>
       <c r="B20" t="s">
+        <v>38</v>
+      </c>
+      <c r="C20" t="s">
         <v>56</v>
-      </c>
-      <c r="C20" t="s">
-        <v>57</v>
       </c>
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B21" t="s">
         <v>33</v>
       </c>
       <c r="C21" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
+        <v>59</v>
+      </c>
+      <c r="B22" t="s">
         <v>60</v>
       </c>
-      <c r="B22" t="s">
+      <c r="C22" t="s">
         <v>61</v>
-      </c>
-      <c r="C22" t="s">
-        <v>62</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
+        <v>62</v>
+      </c>
+      <c r="B23" t="s">
         <v>63</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
         <v>64</v>
-      </c>
-      <c r="C23" t="s">
-        <v>65</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
+        <v>65</v>
+      </c>
+      <c r="B24" t="s">
         <v>66</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>67</v>
-      </c>
-      <c r="C24" t="s">
-        <v>68</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
+        <v>68</v>
+      </c>
+      <c r="B25" t="s">
         <v>69</v>
-      </c>
-      <c r="B25" t="s">
-        <v>38</v>
       </c>
       <c r="C25" t="s">
         <v>70</v>
@@ -2093,7 +2100,7 @@
         <v>71</v>
       </c>
       <c r="B26" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="C26" t="s">
         <v>72</v>
@@ -2104,7 +2111,7 @@
         <v>73</v>
       </c>
       <c r="B27" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="C27" t="s">
         <v>74</v>
@@ -2243,7 +2250,7 @@
         <v>96</v>
       </c>
       <c r="B10" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="C10" t="s">
         <v>97</v>
@@ -2480,7 +2487,7 @@
         <v>145</v>
       </c>
       <c r="G2" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="H2" t="s">
         <v>83</v>
@@ -2498,7 +2505,7 @@
         <v>146</v>
       </c>
       <c r="M2" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -2521,7 +2528,7 @@
         <v>145</v>
       </c>
       <c r="G3" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="H3" t="s">
         <v>83</v>
@@ -2539,7 +2546,7 @@
         <v>149</v>
       </c>
       <c r="M3" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="4" spans="1:13">
@@ -2562,7 +2569,7 @@
         <v>145</v>
       </c>
       <c r="G4" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="H4" t="s">
         <v>83</v>
@@ -2580,7 +2587,7 @@
         <v>149</v>
       </c>
       <c r="M4" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -2603,7 +2610,7 @@
         <v>145</v>
       </c>
       <c r="G5" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="H5" t="s">
         <v>83</v>
@@ -2621,7 +2628,7 @@
         <v>149</v>
       </c>
       <c r="M5" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -2644,7 +2651,7 @@
         <v>145</v>
       </c>
       <c r="G6" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="H6" t="s">
         <v>83</v>
@@ -2662,7 +2669,7 @@
         <v>149</v>
       </c>
       <c r="M6" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -2685,7 +2692,7 @@
         <v>145</v>
       </c>
       <c r="G7" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="H7" t="s">
         <v>83</v>
@@ -2703,7 +2710,7 @@
         <v>149</v>
       </c>
       <c r="M7" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="8" spans="1:13">
@@ -2726,7 +2733,7 @@
         <v>145</v>
       </c>
       <c r="G8" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="H8" t="s">
         <v>83</v>
@@ -2744,7 +2751,7 @@
         <v>149</v>
       </c>
       <c r="M8" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="9" spans="1:13">
@@ -2767,7 +2774,7 @@
         <v>145</v>
       </c>
       <c r="G9" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="H9" t="s">
         <v>83</v>
@@ -2785,7 +2792,7 @@
         <v>149</v>
       </c>
       <c r="M9" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="10" spans="1:13">
@@ -2808,7 +2815,7 @@
         <v>145</v>
       </c>
       <c r="G10" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="H10" t="s">
         <v>83</v>
@@ -2826,7 +2833,7 @@
         <v>149</v>
       </c>
       <c r="M10" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -2849,7 +2856,7 @@
         <v>145</v>
       </c>
       <c r="G11" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="H11" t="s">
         <v>83</v>
@@ -2867,7 +2874,7 @@
         <v>149</v>
       </c>
       <c r="M11" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -2890,7 +2897,7 @@
         <v>145</v>
       </c>
       <c r="G12" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="H12" t="s">
         <v>83</v>
@@ -2908,7 +2915,7 @@
         <v>149</v>
       </c>
       <c r="M12" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -2931,7 +2938,7 @@
         <v>145</v>
       </c>
       <c r="G13" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="H13" t="s">
         <v>83</v>
@@ -2949,7 +2956,7 @@
         <v>160</v>
       </c>
       <c r="M13" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="14" spans="1:13">
@@ -2972,7 +2979,7 @@
         <v>145</v>
       </c>
       <c r="G14" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="H14" t="s">
         <v>83</v>
@@ -2990,7 +2997,7 @@
         <v>160</v>
       </c>
       <c r="M14" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="15" spans="1:13">
@@ -3013,7 +3020,7 @@
         <v>145</v>
       </c>
       <c r="G15" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="H15" t="s">
         <v>83</v>
@@ -3031,7 +3038,7 @@
         <v>160</v>
       </c>
       <c r="M15" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
     <row r="16" spans="1:13">
@@ -3054,7 +3061,7 @@
         <v>145</v>
       </c>
       <c r="G16" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="H16" t="s">
         <v>83</v>
@@ -3072,7 +3079,7 @@
         <v>160</v>
       </c>
       <c r="M16" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
     </row>
   </sheetData>
@@ -3253,7 +3260,7 @@
         <v>191</v>
       </c>
       <c r="B2" t="s">
-        <v>38</v>
+        <v>69</v>
       </c>
       <c r="C2" t="s">
         <v>41</v>
@@ -3271,13 +3278,13 @@
         <v>53</v>
       </c>
       <c r="H2" t="s">
-        <v>56</v>
+        <v>38</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="K2" t="s">
         <v>192</v>

</xml_diff>

<commit_message>
Release v1.1.11-r1: MQTT per-target queues, operator stop persistence, and platform fixes.
Persist manual stop across service restarts; harden installer shutdown when UI is open; add Android acquisition foreground service; improve Windows title bar icon and startup Excel handling.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/config/lines/C型火焰复合机.xlsx
+++ b/config/lines/C型火焰复合机.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="15120" windowHeight="11760"/>
+    <workbookView windowWidth="28800" windowHeight="11775"/>
   </bookViews>
   <sheets>
     <sheet name="配置" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="369" uniqueCount="193">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="195">
   <si>
     <t>配置项</t>
   </si>
@@ -129,10 +129,16 @@
     <t>扫描周期毫秒</t>
   </si>
   <si>
+    <t>ScanIntervalMs</t>
+  </si>
+  <si>
+    <t>发布周期毫秒</t>
+  </si>
+  <si>
     <t>60000</t>
   </si>
   <si>
-    <t>ScanIntervalMs</t>
+    <t>PublishIntervalMs</t>
   </si>
   <si>
     <t>温度发布阈值</t>
@@ -628,7 +634,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="23">
+  <fonts count="24">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -637,6 +643,12 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Calibri"/>
+      <charset val="134"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -1103,155 +1115,156 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
-    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1812,7 +1825,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C28"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="14.4285714285714" customWidth="1"/>
@@ -1934,30 +1947,30 @@
       <c r="A11" t="s">
         <v>29</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11">
+        <v>2000</v>
+      </c>
+      <c r="C11" t="s">
         <v>30</v>
       </c>
-      <c r="C11" t="s">
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" s="2" t="s">
         <v>31</v>
       </c>
-    </row>
-    <row r="12" spans="1:3">
-      <c r="A12" t="s">
+      <c r="B12" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="B12" t="s">
+      <c r="C12" s="2" t="s">
         <v>33</v>
-      </c>
-      <c r="C12" t="s">
-        <v>34</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
+        <v>34</v>
+      </c>
+      <c r="B13" t="s">
         <v>35</v>
-      </c>
-      <c r="B13" t="s">
-        <v>24</v>
       </c>
       <c r="C13" t="s">
         <v>36</v>
@@ -1967,74 +1980,74 @@
       <c r="A14" t="s">
         <v>37</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" t="s">
+        <v>24</v>
+      </c>
+      <c r="C14" t="s">
         <v>38</v>
-      </c>
-      <c r="C14" t="s">
-        <v>39</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
+        <v>39</v>
+      </c>
+      <c r="B15" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="B15" t="s">
+      <c r="C15" t="s">
         <v>41</v>
-      </c>
-      <c r="C15" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" t="s">
         <v>43</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>44</v>
-      </c>
-      <c r="C16" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" t="s">
         <v>46</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C17" t="s">
         <v>47</v>
-      </c>
-      <c r="C17" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" t="s">
         <v>49</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>50</v>
-      </c>
-      <c r="C18" t="s">
-        <v>51</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
+        <v>51</v>
+      </c>
+      <c r="B19" t="s">
         <v>52</v>
       </c>
-      <c r="B19" t="s">
+      <c r="C19" t="s">
         <v>53</v>
-      </c>
-      <c r="C19" t="s">
-        <v>54</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
+        <v>54</v>
+      </c>
+      <c r="B20" t="s">
         <v>55</v>
-      </c>
-      <c r="B20" t="s">
-        <v>38</v>
       </c>
       <c r="C20" t="s">
         <v>56</v>
@@ -2045,7 +2058,7 @@
         <v>57</v>
       </c>
       <c r="B21" t="s">
-        <v>33</v>
+        <v>40</v>
       </c>
       <c r="C21" t="s">
         <v>58</v>
@@ -2056,51 +2069,51 @@
         <v>59</v>
       </c>
       <c r="B22" t="s">
+        <v>35</v>
+      </c>
+      <c r="C22" t="s">
         <v>60</v>
-      </c>
-      <c r="C22" t="s">
-        <v>61</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
+        <v>61</v>
+      </c>
+      <c r="B23" t="s">
         <v>62</v>
       </c>
-      <c r="B23" t="s">
+      <c r="C23" t="s">
         <v>63</v>
-      </c>
-      <c r="C23" t="s">
-        <v>64</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
+        <v>64</v>
+      </c>
+      <c r="B24" t="s">
         <v>65</v>
       </c>
-      <c r="B24" t="s">
+      <c r="C24" t="s">
         <v>66</v>
-      </c>
-      <c r="C24" t="s">
-        <v>67</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
+        <v>67</v>
+      </c>
+      <c r="B25" t="s">
         <v>68</v>
       </c>
-      <c r="B25" t="s">
+      <c r="C25" t="s">
         <v>69</v>
-      </c>
-      <c r="C25" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
+        <v>70</v>
+      </c>
+      <c r="B26" t="s">
         <v>71</v>
-      </c>
-      <c r="B26" t="s">
-        <v>69</v>
       </c>
       <c r="C26" t="s">
         <v>72</v>
@@ -2111,7 +2124,7 @@
         <v>73</v>
       </c>
       <c r="B27" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C27" t="s">
         <v>74</v>
@@ -2121,11 +2134,22 @@
       <c r="A28" t="s">
         <v>75</v>
       </c>
-      <c r="B28">
-        <v>1</v>
+      <c r="B28" t="s">
+        <v>71</v>
       </c>
       <c r="C28" t="s">
         <v>76</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" t="s">
+        <v>77</v>
+      </c>
+      <c r="B29">
+        <v>1</v>
+      </c>
+      <c r="C29" t="s">
+        <v>78</v>
       </c>
     </row>
   </sheetData>
@@ -2159,101 +2183,101 @@
     </row>
     <row r="2" spans="1:3">
       <c r="A2" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="B2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C2" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:3">
       <c r="A3" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="B3" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C3" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
     </row>
     <row r="4" spans="1:3">
       <c r="A4" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="B4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C4" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:3">
       <c r="A5" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="B5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C5" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" spans="1:3">
       <c r="A6" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="B6" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C6" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="B7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C7" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="B8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C8" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
     </row>
     <row r="9" spans="1:3">
       <c r="A9" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="B9" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C9" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="B10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C10" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
     </row>
   </sheetData>
@@ -2275,130 +2299,130 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:2">
       <c r="A1" s="1" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="B2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="B3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="B4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="B5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="B6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="B7" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="B8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="B9" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="B10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="B11" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="B12" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="B13" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="B14" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="B15" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="B16" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -2428,72 +2452,72 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:13">
       <c r="A1" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:13">
       <c r="A2" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="B2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C2" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D2" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="E2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F2" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I2" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="J2">
         <v>1</v>
@@ -2502,39 +2526,39 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="M2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="3" spans="1:13">
       <c r="A3" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="B3" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C3" t="s">
+        <v>149</v>
+      </c>
+      <c r="D3" t="s">
+        <v>150</v>
+      </c>
+      <c r="E3" t="s">
+        <v>85</v>
+      </c>
+      <c r="F3" t="s">
         <v>147</v>
       </c>
-      <c r="D3" t="s">
-        <v>148</v>
-      </c>
-      <c r="E3" t="s">
-        <v>83</v>
-      </c>
-      <c r="F3" t="s">
-        <v>145</v>
-      </c>
       <c r="G3" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I3" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="J3">
         <v>1</v>
@@ -2543,39 +2567,39 @@
         <v>0</v>
       </c>
       <c r="L3" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="M3" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="B4" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C4" t="s">
+        <v>152</v>
+      </c>
+      <c r="D4" t="s">
         <v>150</v>
       </c>
-      <c r="D4" t="s">
-        <v>148</v>
-      </c>
       <c r="E4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F4" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I4" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="J4">
         <v>1</v>
@@ -2584,39 +2608,39 @@
         <v>0</v>
       </c>
       <c r="L4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="M4" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="5" spans="1:13">
       <c r="A5" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="B5" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C5" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D5" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F5" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I5" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="J5">
         <v>1</v>
@@ -2625,39 +2649,39 @@
         <v>0</v>
       </c>
       <c r="L5" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="M5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="6" spans="1:13">
       <c r="A6" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="B6" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C6" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="D6" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F6" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I6" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="J6">
         <v>1</v>
@@ -2666,39 +2690,39 @@
         <v>0</v>
       </c>
       <c r="L6" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="M6" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="7" spans="1:13">
       <c r="A7" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="B7" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C7" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D7" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F7" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I7" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="J7">
         <v>1</v>
@@ -2707,39 +2731,39 @@
         <v>0</v>
       </c>
       <c r="L7" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="M7" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="B8" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C8" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="D8" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F8" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="J8">
         <v>1</v>
@@ -2748,39 +2772,39 @@
         <v>0</v>
       </c>
       <c r="L8" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="M8" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="B9" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C9" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D9" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E9" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F9" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G9" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H9" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I9" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="J9">
         <v>1</v>
@@ -2789,39 +2813,39 @@
         <v>0</v>
       </c>
       <c r="L9" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="M9" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="10" spans="1:13">
       <c r="A10" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="B10" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C10" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="D10" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F10" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G10" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I10" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="J10">
         <v>1</v>
@@ -2830,39 +2854,39 @@
         <v>0</v>
       </c>
       <c r="L10" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="M10" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="11" spans="1:13">
       <c r="A11" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="B11" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C11" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D11" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E11" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F11" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H11" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I11" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="J11">
         <v>1</v>
@@ -2871,39 +2895,39 @@
         <v>0</v>
       </c>
       <c r="L11" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="M11" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="12" spans="1:13">
       <c r="A12" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="B12" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="C12" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="D12" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E12" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F12" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G12" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H12" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I12" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="J12">
         <v>1</v>
@@ -2912,39 +2936,39 @@
         <v>0</v>
       </c>
       <c r="L12" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="M12" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="13" spans="1:13">
       <c r="A13" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="B13" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C13" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D13" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E13" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F13" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G13" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H13" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I13" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="J13">
         <v>1</v>
@@ -2953,39 +2977,39 @@
         <v>0</v>
       </c>
       <c r="L13" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="M13" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="14" spans="1:13">
       <c r="A14" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="B14" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C14" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D14" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E14" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F14" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G14" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H14" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I14" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="J14">
         <v>1</v>
@@ -2994,39 +3018,39 @@
         <v>0</v>
       </c>
       <c r="L14" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="M14" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="15" spans="1:13">
       <c r="A15" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="B15" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C15" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D15" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E15" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F15" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G15" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H15" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I15" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="J15">
         <v>1</v>
@@ -3035,39 +3059,39 @@
         <v>0</v>
       </c>
       <c r="L15" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="M15" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
     <row r="16" spans="1:13">
       <c r="A16" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
       <c r="B16" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="C16" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D16" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="E16" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="F16" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="G16" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H16" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="I16" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="J16">
         <v>1</v>
@@ -3076,10 +3100,10 @@
         <v>0</v>
       </c>
       <c r="L16" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="M16" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
     </row>
   </sheetData>
@@ -3103,96 +3127,96 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B2" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="C2" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="D2" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>166</v>
+        <v>168</v>
       </c>
       <c r="B3" t="s">
-        <v>167</v>
+        <v>169</v>
       </c>
       <c r="C3" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="D3" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="B4" t="s">
-        <v>170</v>
+        <v>172</v>
       </c>
       <c r="C4" t="s">
-        <v>171</v>
+        <v>173</v>
       </c>
       <c r="D4" t="s">
-        <v>172</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="B5" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="C5" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="D5" t="s">
-        <v>175</v>
+        <v>177</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>176</v>
+        <v>178</v>
       </c>
       <c r="B6" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="C6" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="D6" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>180</v>
+        <v>182</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
     </row>
   </sheetData>
@@ -3222,72 +3246,72 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:11">
       <c r="A1" s="1" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D2">
         <v>1888</v>
       </c>
       <c r="E2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="G2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="H2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="I2">
         <v>0</v>
       </c>
       <c r="J2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="K2" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Release v1.1.14: isolated Windows hosts, subscribe-by-sender catalog, and faster sub-instance startup.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/config/lines/C型火焰复合机.xlsx
+++ b/config/lines/C型火焰复合机.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="28800" windowHeight="11775"/>
+    <workbookView windowWidth="23040" windowHeight="12360" activeTab="3"/>
   </bookViews>
   <sheets>
     <sheet name="配置" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="371" uniqueCount="195">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="343" uniqueCount="188">
   <si>
     <t>配置项</t>
   </si>
@@ -375,18 +375,6 @@
     <t>下夹距</t>
   </si>
   <si>
-    <t>shkjjl</t>
-  </si>
-  <si>
-    <t>上火口距离</t>
-  </si>
-  <si>
-    <t>xhkjjl</t>
-  </si>
-  <si>
-    <t>下火口距离</t>
-  </si>
-  <si>
     <t>smqll</t>
   </si>
   <si>
@@ -504,16 +492,7 @@
     <t>D1040</t>
   </si>
   <si>
-    <t>D1050</t>
-  </si>
-  <si>
-    <t>D1060</t>
-  </si>
-  <si>
-    <t>D1070</t>
-  </si>
-  <si>
-    <t>D1080</t>
+    <t>手动</t>
   </si>
   <si>
     <t>D1090</t>
@@ -522,7 +501,7 @@
     <t>D1100</t>
   </si>
   <si>
-    <t>手动</t>
+    <t>D1110</t>
   </si>
   <si>
     <t>设定参数</t>
@@ -634,7 +613,7 @@
     <numFmt numFmtId="43" formatCode="_ * #,##0.00_ ;_ * \-#,##0.00_ ;_ * &quot;-&quot;??_ ;_ @_ "/>
     <numFmt numFmtId="44" formatCode="_ &quot;￥&quot;* #,##0.00_ ;_ &quot;￥&quot;* \-#,##0.00_ ;_ &quot;￥&quot;* &quot;-&quot;??_ ;_ @_ "/>
   </numFmts>
-  <fonts count="24">
+  <fonts count="23">
     <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
@@ -643,12 +622,6 @@
     </font>
     <font>
       <b/>
-      <sz val="11"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <charset val="134"/>
-    </font>
-    <font>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
@@ -1115,148 +1088,148 @@
   </borders>
   <cellStyleXfs count="49">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyBorder="0"/>
-    <xf numFmtId="43" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="44" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="41" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="42" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="43" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="44" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="41" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="42" fontId="3" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="2" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="19" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="3" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="5" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="4" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="5" borderId="6" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="7" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="8" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="9" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="10" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="11" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="12" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
@@ -1264,7 +1237,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1" applyProtection="1"/>
   </cellXfs>
   <cellStyles count="49">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -1955,13 +1928,13 @@
       </c>
     </row>
     <row r="12" spans="1:3">
-      <c r="A12" s="2" t="s">
+      <c r="A12" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="3" t="s">
         <v>33</v>
       </c>
     </row>
@@ -1991,7 +1964,7 @@
       <c r="A15" t="s">
         <v>39</v>
       </c>
-      <c r="B15" s="3" t="s">
+      <c r="B15" s="2" t="s">
         <v>40</v>
       </c>
       <c r="C15" t="s">
@@ -2290,7 +2263,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15" outlineLevelCol="1"/>
   <cols>
     <col min="1" max="1" width="10.5714285714286" customWidth="1"/>
@@ -2407,22 +2380,6 @@
       </c>
       <c r="B14" t="s">
         <v>127</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2">
-      <c r="A15" t="s">
-        <v>128</v>
-      </c>
-      <c r="B15" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="16" spans="1:2">
-      <c r="A16" t="s">
-        <v>130</v>
-      </c>
-      <c r="B16" t="s">
-        <v>131</v>
       </c>
     </row>
   </sheetData>
@@ -2435,11 +2392,11 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:M16"/>
+  <dimension ref="A1:M14"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="7.28571428571429" customWidth="1"/>
-    <col min="2" max="2" width="4.14285714285714" customWidth="1"/>
+    <col min="1" max="1" width="23.4285714285714" customWidth="1"/>
+    <col min="2" max="2" width="14.1428571428571" customWidth="1"/>
     <col min="3" max="3" width="6.28571428571429" customWidth="1"/>
     <col min="4" max="4" width="7.57142857142857" customWidth="1"/>
     <col min="5" max="5" width="3" customWidth="1"/>
@@ -2452,43 +2409,43 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:13">
       <c r="A1" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>130</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>132</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>133</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>134</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="H1" s="1" t="s">
         <v>135</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>136</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>137</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>138</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>139</v>
       </c>
       <c r="I1" s="1" t="s">
         <v>37</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>141</v>
+        <v>137</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>143</v>
+        <v>139</v>
       </c>
     </row>
     <row r="2" spans="1:13">
@@ -2496,19 +2453,19 @@
         <v>103</v>
       </c>
       <c r="B2" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C2" t="s">
-        <v>145</v>
+        <v>141</v>
       </c>
       <c r="D2" t="s">
-        <v>146</v>
+        <v>142</v>
       </c>
       <c r="E2" t="s">
         <v>85</v>
       </c>
       <c r="F2" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="G2" t="s">
         <v>71</v>
@@ -2526,7 +2483,7 @@
         <v>0</v>
       </c>
       <c r="L2" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="M2" t="s">
         <v>40</v>
@@ -2537,19 +2494,19 @@
         <v>105</v>
       </c>
       <c r="B3" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C3" t="s">
-        <v>149</v>
+        <v>145</v>
       </c>
       <c r="D3" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E3" t="s">
         <v>85</v>
       </c>
       <c r="F3" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="G3" t="s">
         <v>71</v>
@@ -2567,7 +2524,7 @@
         <v>0</v>
       </c>
       <c r="L3" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="M3" t="s">
         <v>40</v>
@@ -2578,19 +2535,19 @@
         <v>107</v>
       </c>
       <c r="B4" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C4" t="s">
-        <v>152</v>
+        <v>148</v>
       </c>
       <c r="D4" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E4" t="s">
         <v>85</v>
       </c>
       <c r="F4" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="G4" t="s">
         <v>71</v>
@@ -2608,7 +2565,7 @@
         <v>0</v>
       </c>
       <c r="L4" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="M4" t="s">
         <v>40</v>
@@ -2619,19 +2576,19 @@
         <v>109</v>
       </c>
       <c r="B5" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C5" t="s">
-        <v>153</v>
+        <v>149</v>
       </c>
       <c r="D5" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E5" t="s">
         <v>85</v>
       </c>
       <c r="F5" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="G5" t="s">
         <v>71</v>
@@ -2649,7 +2606,7 @@
         <v>0</v>
       </c>
       <c r="L5" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="M5" t="s">
         <v>40</v>
@@ -2660,19 +2617,19 @@
         <v>111</v>
       </c>
       <c r="B6" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C6" t="s">
-        <v>154</v>
+        <v>150</v>
       </c>
       <c r="D6" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E6" t="s">
         <v>85</v>
       </c>
       <c r="F6" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="G6" t="s">
         <v>71</v>
@@ -2690,7 +2647,7 @@
         <v>0</v>
       </c>
       <c r="L6" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="M6" t="s">
         <v>40</v>
@@ -2700,20 +2657,17 @@
       <c r="A7" t="s">
         <v>113</v>
       </c>
-      <c r="B7" t="s">
-        <v>144</v>
-      </c>
-      <c r="C7" t="s">
-        <v>155</v>
+      <c r="B7" s="2" t="s">
+        <v>151</v>
       </c>
       <c r="D7" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E7" t="s">
         <v>85</v>
       </c>
       <c r="F7" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="G7" t="s">
         <v>71</v>
@@ -2731,7 +2685,7 @@
         <v>0</v>
       </c>
       <c r="L7" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="M7" t="s">
         <v>40</v>
@@ -2741,20 +2695,17 @@
       <c r="A8" t="s">
         <v>115</v>
       </c>
-      <c r="B8" t="s">
-        <v>144</v>
-      </c>
-      <c r="C8" t="s">
-        <v>156</v>
+      <c r="B8" s="2" t="s">
+        <v>151</v>
       </c>
       <c r="D8" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E8" t="s">
         <v>85</v>
       </c>
       <c r="F8" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="G8" t="s">
         <v>71</v>
@@ -2772,7 +2723,7 @@
         <v>0</v>
       </c>
       <c r="L8" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="M8" t="s">
         <v>40</v>
@@ -2783,19 +2734,19 @@
         <v>117</v>
       </c>
       <c r="B9" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C9" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="D9" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E9" t="s">
         <v>85</v>
       </c>
       <c r="F9" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="G9" t="s">
         <v>71</v>
@@ -2813,7 +2764,7 @@
         <v>0</v>
       </c>
       <c r="L9" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="M9" t="s">
         <v>40</v>
@@ -2824,19 +2775,19 @@
         <v>119</v>
       </c>
       <c r="B10" t="s">
-        <v>144</v>
+        <v>140</v>
       </c>
       <c r="C10" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="D10" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E10" t="s">
         <v>85</v>
       </c>
       <c r="F10" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="G10" t="s">
         <v>71</v>
@@ -2854,7 +2805,7 @@
         <v>0</v>
       </c>
       <c r="L10" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="M10" t="s">
         <v>40</v>
@@ -2864,20 +2815,20 @@
       <c r="A11" t="s">
         <v>121</v>
       </c>
-      <c r="B11" t="s">
-        <v>144</v>
+      <c r="B11" s="2" t="s">
+        <v>140</v>
       </c>
       <c r="C11" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="D11" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E11" t="s">
         <v>85</v>
       </c>
       <c r="F11" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="G11" t="s">
         <v>71</v>
@@ -2895,7 +2846,7 @@
         <v>0</v>
       </c>
       <c r="L11" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="M11" t="s">
         <v>40</v>
@@ -2906,19 +2857,19 @@
         <v>123</v>
       </c>
       <c r="B12" t="s">
-        <v>144</v>
+        <v>151</v>
       </c>
       <c r="C12" t="s">
-        <v>160</v>
+        <v>85</v>
       </c>
       <c r="D12" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E12" t="s">
         <v>85</v>
       </c>
       <c r="F12" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="G12" t="s">
         <v>71</v>
@@ -2936,7 +2887,7 @@
         <v>0</v>
       </c>
       <c r="L12" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="M12" t="s">
         <v>40</v>
@@ -2947,19 +2898,19 @@
         <v>125</v>
       </c>
       <c r="B13" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="C13" t="s">
         <v>85</v>
       </c>
       <c r="D13" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E13" t="s">
         <v>85</v>
       </c>
       <c r="F13" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="G13" t="s">
         <v>71</v>
@@ -2977,7 +2928,7 @@
         <v>0</v>
       </c>
       <c r="L13" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="M13" t="s">
         <v>40</v>
@@ -2988,19 +2939,19 @@
         <v>127</v>
       </c>
       <c r="B14" t="s">
-        <v>161</v>
+        <v>151</v>
       </c>
       <c r="C14" t="s">
         <v>85</v>
       </c>
       <c r="D14" t="s">
-        <v>150</v>
+        <v>146</v>
       </c>
       <c r="E14" t="s">
         <v>85</v>
       </c>
       <c r="F14" t="s">
-        <v>147</v>
+        <v>143</v>
       </c>
       <c r="G14" t="s">
         <v>71</v>
@@ -3018,91 +2969,9 @@
         <v>0</v>
       </c>
       <c r="L14" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="M14" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13">
-      <c r="A15" t="s">
-        <v>129</v>
-      </c>
-      <c r="B15" t="s">
-        <v>161</v>
-      </c>
-      <c r="C15" t="s">
-        <v>85</v>
-      </c>
-      <c r="D15" t="s">
-        <v>150</v>
-      </c>
-      <c r="E15" t="s">
-        <v>85</v>
-      </c>
-      <c r="F15" t="s">
-        <v>147</v>
-      </c>
-      <c r="G15" t="s">
-        <v>71</v>
-      </c>
-      <c r="H15" t="s">
-        <v>85</v>
-      </c>
-      <c r="I15" t="s">
-        <v>85</v>
-      </c>
-      <c r="J15">
-        <v>1</v>
-      </c>
-      <c r="K15">
-        <v>0</v>
-      </c>
-      <c r="L15" t="s">
-        <v>162</v>
-      </c>
-      <c r="M15" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13">
-      <c r="A16" t="s">
-        <v>131</v>
-      </c>
-      <c r="B16" t="s">
-        <v>161</v>
-      </c>
-      <c r="C16" t="s">
-        <v>85</v>
-      </c>
-      <c r="D16" t="s">
-        <v>150</v>
-      </c>
-      <c r="E16" t="s">
-        <v>85</v>
-      </c>
-      <c r="F16" t="s">
-        <v>147</v>
-      </c>
-      <c r="G16" t="s">
-        <v>71</v>
-      </c>
-      <c r="H16" t="s">
-        <v>85</v>
-      </c>
-      <c r="I16" t="s">
-        <v>85</v>
-      </c>
-      <c r="J16">
-        <v>1</v>
-      </c>
-      <c r="K16">
-        <v>0</v>
-      </c>
-      <c r="L16" t="s">
-        <v>162</v>
-      </c>
-      <c r="M16" t="s">
         <v>40</v>
       </c>
     </row>
@@ -3127,96 +2996,96 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="B1" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>163</v>
+        <v>156</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" t="s">
-        <v>148</v>
+        <v>144</v>
       </c>
       <c r="B2" t="s">
-        <v>165</v>
+        <v>158</v>
       </c>
       <c r="C2" t="s">
-        <v>166</v>
+        <v>159</v>
       </c>
       <c r="D2" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="B3" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="C3" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="D3" t="s">
-        <v>171</v>
+        <v>164</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" t="s">
-        <v>151</v>
+        <v>147</v>
       </c>
       <c r="B4" t="s">
-        <v>172</v>
+        <v>165</v>
       </c>
       <c r="C4" t="s">
-        <v>173</v>
+        <v>166</v>
       </c>
       <c r="D4" t="s">
-        <v>174</v>
+        <v>167</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" t="s">
-        <v>162</v>
+        <v>155</v>
       </c>
       <c r="B5" t="s">
-        <v>175</v>
+        <v>168</v>
       </c>
       <c r="C5" t="s">
-        <v>176</v>
+        <v>169</v>
       </c>
       <c r="D5" t="s">
-        <v>177</v>
+        <v>170</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" t="s">
-        <v>178</v>
+        <v>171</v>
       </c>
       <c r="B6" t="s">
-        <v>179</v>
+        <v>172</v>
       </c>
       <c r="C6" t="s">
-        <v>180</v>
+        <v>173</v>
       </c>
       <c r="D6" t="s">
-        <v>181</v>
+        <v>174</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" t="s">
-        <v>182</v>
+        <v>175</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" t="s">
-        <v>183</v>
+        <v>176</v>
       </c>
     </row>
   </sheetData>
@@ -3246,42 +3115,42 @@
   <sheetData>
     <row r="1" s="1" customFormat="1" spans="1:11">
       <c r="A1" s="1" t="s">
-        <v>132</v>
+        <v>128</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>138</v>
+        <v>134</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>177</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>178</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>179</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>180</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>181</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>182</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>183</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="K1" s="1" t="s">
         <v>185</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>186</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>187</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>188</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>189</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>190</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>191</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="2" spans="1:11">
       <c r="A2" t="s">
-        <v>193</v>
+        <v>186</v>
       </c>
       <c r="B2" t="s">
         <v>71</v>
@@ -3311,7 +3180,7 @@
         <v>62</v>
       </c>
       <c r="K2" t="s">
-        <v>194</v>
+        <v>187</v>
       </c>
     </row>
   </sheetData>

</xml_diff>